<commit_message>
Reorganize Ingresos filters (Cliente/Tipo arriba, pestaña Hoy, mensuales vigentes)
Los filtros de Cliente y Tipo de pago ahora aparecen por encima de las
pestañas de fecha (Hoy/Esta Semana/Historial/Estadísticas). Al filtrar
por Tipo = Mensual se muestran solo los pagos vigentes con órdenes
disponibles, igual criterio que usa el asistente de pedidos para
ofrecer un pago reutilizable. Actualiza RF-44/RF-67 y el mapa técnico.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Requerimientos_Oasis.xlsx
+++ b/docs/Requerimientos_Oasis.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2232,7 +2232,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-08-17, a petición del usuario] Se reordenó la jerarquía de filtros: Cliente y Tipo de pago ahora son el filtro principal, mostrado por encima de las pestañas de fecha (antes al revés). Se agregó una pestaña 'Hoy' (antes solo Esta Semana/Historial), quedando Hoy / Esta Semana / Historial / Estadísticas. Ver también RF-67 (filtro de mensuales vigentes).</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -3029,6 +3033,43 @@
       <c r="G70" s="8" t="inlineStr">
         <is>
           <t>[Nuevo 2026-07-31, a petición del usuario] Implementado con un modelo de cantidades (no on/off): cada ítem tiene un stepper +/- (ComboCategorySelector.jsx) en vez de un checkbox, así que puede elegirse el mismo ítem varias veces. Al llegar al máximo configurado (de su categoría o del pool Arroz/Proteína/Acompañamiento/Extra), cada nueva unidad abre un modal (ComboExtraChargeModal.jsx) que avisa que es un extra y pide su precio, precargado con el último monto usado para ese ítem — se puede repetir para agregar tantas unidades extra como haga falta, del mismo ítem o de varios, cada una con su propio precio. Lógica de cantidades/extras centralizada en el hook useComboSelections.js (src/hooks); cada unidad se persiste como una fila propia en combo_order_selections (is_extra/extra_charge, migración 20260731_combo_order_selections_extra.sql — mismo criterio que ya usa aggregateComboSelections para contar producción, sin necesidad de columna de cantidad). El precio total (computeComboPrice) y los resúmenes (paso de confirmación, ComboOrderCard) agrupan esas filas por ítem con groupSelectionsByItem para mostrar 'Ítem ×N' y el desglose de extras. Pendiente de aplicar en la base de datos real: la migración SQL no se ejecutó contra Supabase en esta sesión (no había credenciales/CLI vinculado disponibles). No se pudo probar end-to-end con Playwright contra el entorno real por la misma razón — sí se verificó que build y lint pasan sin errores nuevos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>RF-67</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Pagos y Facturación</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Filtrar pagos mensuales vigentes con cupo disponible</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Al filtrar Ingresos por Tipo de pago = 'Mensual', el sistema debe mostrar únicamente los pagos mensuales vigentes (no cerrados manualmente, no cancelados) que todavía tienen cupo (menos de 4 órdenes vinculadas) — el mismo criterio de elegibilidad que usa el asistente de pedidos para ofrecer un pago reutilizable — en vez de listar también los ya completos, cerrados o cancelados.</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-08-17, a petición del usuario] Payments.jsx: filtro de Tipo de pago, al valor 'monthly', además de igualar payment_type aplica status in (pending, paid) AND closed_at IS NULL AND órdenes vinculadas &lt; 4, con un badge visible ('Mostrando solo mensuales vigentes con órdenes disponibles'). Pensado para auditar de un vistazo cuál es el pago mensual activo de cada cliente y detectar fragmentación (más de un pago vigente simultáneo para el mismo cliente) sin consultar la base de datos directamente — ver project-monthly-payment-fragmentation en memoria. Verificado con Playwright contra producción: con este filtro + pestaña Historial se confirmaron 11 pagos mensuales vigentes, uno por cliente, sin duplicados; el filtro destapó un pago suelto real (Erick Vásquez #19, 2/4, de junio) que se había quedado sin cerrar en una limpieza de datos anterior — se cerró en el momento.</t>
         </is>
       </c>
     </row>

</xml_diff>